<commit_message>
update table 1 output
</commit_message>
<xml_diff>
--- a/CPRD Raw Analysis/Results/Table1_Raw.xlsx
+++ b/CPRD Raw Analysis/Results/Table1_Raw.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -400,7 +400,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Vertical</t>
+          <t>Vertebral</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -581,6 +581,18 @@
       <c r="B20" t="inlineStr">
         <is>
           <t>74 (0.3%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Follow up time</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>730 days (709 days, 730 days)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
update the Raw analysis files
</commit_message>
<xml_diff>
--- a/CPRD Raw Analysis/Results/Table1_Raw.xlsx
+++ b/CPRD Raw Analysis/Results/Table1_Raw.xlsx
@@ -369,7 +369,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Age at fracture occurrence</t>
+          <t>Age at Fracture Occurrence</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -381,7 +381,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Fracture site</t>
+          <t>Fracture Site</t>
         </is>
       </c>
     </row>
@@ -424,110 +424,110 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Censoring event</t>
+          <t>Censoring Event</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Cancer</t>
+          <t>Max of 730 days from index date</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>552 (2.2%)</t>
+          <t>18,726 (74%)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Cancer, Fracture ensuing incident (index) fracture</t>
+          <t>End of data collection period</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>1 (&lt;0.1%)</t>
+          <t>2,267 (9.0%)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Death</t>
+          <t>Fracture ensuing incident (index) fracture</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>1,695 (6.7%)</t>
+          <t>1,815 (7.2%)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>End of data collection period</t>
+          <t>Death</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2,267 (9.0%)</t>
+          <t>1,695 (6.7%)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>End of data collection period, Cancer</t>
+          <t>Cancer</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>1 (&lt;0.1%)</t>
+          <t>552 (2.2%)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>End of data collection period, Fracture ensuing incident (index) fracture</t>
+          <t>Paget’s disease of the bone, or other metabolic bone diseases</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>1 (&lt;0.1%)</t>
+          <t>74 (0.3%)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Fracture ensuing incident (index) fracture</t>
+          <t>Max of 730 days from index date, End of data collection period</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>1,815 (7.2%)</t>
+          <t>3 (&lt;0.1%)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Max of 730 days from index date</t>
+          <t>Cancer, Fracture ensuing incident (index) fracture</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>18,726 (74%)</t>
+          <t>1 (&lt;0.1%)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Max of 730 days from index date, Cancer</t>
+          <t>End of data collection period, Cancer</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -539,19 +539,19 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Max of 730 days from index date, End of data collection period</t>
+          <t>End of data collection period, Fracture ensuing incident (index) fracture</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>3 (&lt;0.1%)</t>
+          <t>1 (&lt;0.1%)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Max of 730 days from index date, Fracture ensuing incident (index) fracture</t>
+          <t>Max of 730 days from index date, Cancer</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -563,7 +563,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Max of 730 days from index date, Paget’s disease of the bone, or other metabolic bone diseases</t>
+          <t>Max of 730 days from index date, Fracture ensuing incident (index) fracture</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -575,19 +575,19 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Paget’s disease of the bone, or other metabolic bone diseases</t>
+          <t>Max of 730 days from index date, Paget’s disease of the bone, or other metabolic bone diseases</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>74 (0.3%)</t>
+          <t>1 (&lt;0.1%)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Follow up time</t>
+          <t>Follow up Time</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -599,7 +599,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>User status</t>
+          <t>User Status</t>
         </is>
       </c>
     </row>
@@ -630,7 +630,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Non-visits status</t>
+          <t>Non-user Visit Status</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
update and add tables and plots output
</commit_message>
<xml_diff>
--- a/CPRD Raw Analysis/Results/Table1_Raw.xlsx
+++ b/CPRD Raw Analysis/Results/Table1_Raw.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B27"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -587,7 +587,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Follow up time</t>
+          <t>Follow up Time</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -599,7 +599,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Heathcare Service User Status</t>
+          <t>User Status</t>
         </is>
       </c>
     </row>
@@ -630,31 +630,19 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Heathcare Service Non-user Visit Status</t>
+          <t>Non-user Visit Status</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Unknown Visits</t>
+          <t>Visits with Non-clinically Relevant Staff</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2 (0.5%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Visits with Non-clinically Relevant Staff</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>382 (99%)</t>
+          <t>384 (100%)</t>
         </is>
       </c>
     </row>

</xml_diff>